<commit_message>
macro var auto updated
</commit_message>
<xml_diff>
--- a/Input/DLEU/macro_vars_new.xlsx
+++ b/Input/DLEU/macro_vars_new.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,679 +447,681 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1954</v>
+        <v>1955</v>
       </c>
       <c r="B2" t="n">
-        <v>15.29800033569336</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
+        <v>15.55799961090088</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1208543628454208</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1955</v>
+        <v>1956</v>
       </c>
       <c r="B3" t="n">
-        <v>15.55799961090088</v>
+        <v>16.09000015258789</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1208543628454208</v>
+        <v>0.1130886673927307</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1956</v>
+        <v>1957</v>
       </c>
       <c r="B4" t="n">
-        <v>16.09000015258789</v>
+        <v>16.625</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1130886673927307</v>
+        <v>0.1177995428442955</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1957</v>
+        <v>1958</v>
       </c>
       <c r="B5" t="n">
-        <v>16.625</v>
+        <v>17</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1177995428442955</v>
+        <v>0.1131686121225357</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1958</v>
+        <v>1959</v>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>17.23699951171875</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1131686121225357</v>
+        <v>0.1391088515520096</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="B7" t="n">
-        <v>17.23699951171875</v>
+        <v>17.47699928283691</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1391088515520096</v>
+        <v>0.1382348090410233</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1960</v>
+        <v>1961</v>
       </c>
       <c r="B8" t="n">
-        <v>17.47699928283691</v>
+        <v>17.66799926757812</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1382348090410233</v>
+        <v>0.1286213546991348</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1961</v>
+        <v>1962</v>
       </c>
       <c r="B9" t="n">
-        <v>17.66799926757812</v>
+        <v>17.88599967956543</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1286213546991348</v>
+        <v>0.1347446143627167</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1962</v>
+        <v>1963</v>
       </c>
       <c r="B10" t="n">
-        <v>17.88599967956543</v>
+        <v>18.08699989318848</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1347446143627167</v>
+        <v>0.1405454874038696</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1963</v>
+        <v>1964</v>
       </c>
       <c r="B11" t="n">
-        <v>18.08699989318848</v>
+        <v>18.36499977111816</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1405454874038696</v>
+        <v>0.1395965218544006</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1964</v>
+        <v>1965</v>
       </c>
       <c r="B12" t="n">
-        <v>18.36499977111816</v>
+        <v>18.70000076293945</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1395965218544006</v>
+        <v>0.142483726143837</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1965</v>
+        <v>1966</v>
       </c>
       <c r="B13" t="n">
-        <v>18.70000076293945</v>
+        <v>19.22599983215332</v>
       </c>
       <c r="C13" t="n">
-        <v>0.142483726143837</v>
+        <v>0.1429800391197205</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1966</v>
+        <v>1967</v>
       </c>
       <c r="B14" t="n">
-        <v>19.22599983215332</v>
+        <v>19.78499984741211</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1429800391197205</v>
+        <v>0.1331247836351395</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1967</v>
+        <v>1968</v>
       </c>
       <c r="B15" t="n">
-        <v>19.78499984741211</v>
+        <v>20.625</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1331247836351395</v>
+        <v>0.1341102570295334</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1968</v>
+        <v>1969</v>
       </c>
       <c r="B16" t="n">
-        <v>20.625</v>
+        <v>21.64200019836426</v>
       </c>
       <c r="C16" t="n">
-        <v>0.1341102570295334</v>
+        <v>0.1527325659990311</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1969</v>
+        <v>1970</v>
       </c>
       <c r="B17" t="n">
-        <v>21.64200019836426</v>
+        <v>22.78499984741211</v>
       </c>
       <c r="C17" t="n">
-        <v>0.1527325659990311</v>
+        <v>0.1389943808317184</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1970</v>
+        <v>1971</v>
       </c>
       <c r="B18" t="n">
-        <v>22.78499984741211</v>
+        <v>23.94000053405762</v>
       </c>
       <c r="C18" t="n">
-        <v>0.1389943808317184</v>
+        <v>0.1159170567989349</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1971</v>
+        <v>1972</v>
       </c>
       <c r="B19" t="n">
-        <v>23.94000053405762</v>
+        <v>24.97299957275391</v>
       </c>
       <c r="C19" t="n">
-        <v>0.1159170567989349</v>
+        <v>0.1211588308215141</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1972</v>
+        <v>1973</v>
       </c>
       <c r="B20" t="n">
-        <v>24.97299957275391</v>
+        <v>26.33499908447266</v>
       </c>
       <c r="C20" t="n">
-        <v>0.1211588308215141</v>
+        <v>0.1527361124753952</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1973</v>
+        <v>1974</v>
       </c>
       <c r="B21" t="n">
-        <v>26.33499908447266</v>
+        <v>28.70800018310547</v>
       </c>
       <c r="C21" t="n">
-        <v>0.1527361124753952</v>
+        <v>0.1349167227745056</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1974</v>
+        <v>1975</v>
       </c>
       <c r="B22" t="n">
-        <v>28.70800018310547</v>
+        <v>31.35300064086914</v>
       </c>
       <c r="C22" t="n">
-        <v>0.1349167227745056</v>
+        <v>0.08610706031322479</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="B23" t="n">
-        <v>31.35300064086914</v>
+        <v>33.07899856567383</v>
       </c>
       <c r="C23" t="n">
-        <v>0.08610706031322479</v>
+        <v>0.1153995171189308</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1976</v>
+        <v>1977</v>
       </c>
       <c r="B24" t="n">
-        <v>33.07899856567383</v>
+        <v>35.12699890136719</v>
       </c>
       <c r="C24" t="n">
-        <v>0.1153995171189308</v>
+        <v>0.1134625896811485</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1977</v>
+        <v>1978</v>
       </c>
       <c r="B25" t="n">
-        <v>35.12699890136719</v>
+        <v>37.58499908447266</v>
       </c>
       <c r="C25" t="n">
-        <v>0.1134625896811485</v>
+        <v>0.1293336600065231</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1978</v>
+        <v>1979</v>
       </c>
       <c r="B26" t="n">
-        <v>37.58499908447266</v>
+        <v>40.70199966430664</v>
       </c>
       <c r="C26" t="n">
-        <v>0.1293336600065231</v>
+        <v>0.1490096300840378</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1979</v>
+        <v>1980</v>
       </c>
       <c r="B27" t="n">
-        <v>40.70199966430664</v>
+        <v>44.37799835205078</v>
       </c>
       <c r="C27" t="n">
-        <v>0.1490096300840378</v>
+        <v>0.1632433831691742</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1980</v>
+        <v>1981</v>
       </c>
       <c r="B28" t="n">
-        <v>44.37799835205078</v>
+        <v>48.52199935913086</v>
       </c>
       <c r="C28" t="n">
-        <v>0.1632433831691742</v>
+        <v>0.1904037147760391</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1981</v>
+        <v>1982</v>
       </c>
       <c r="B29" t="n">
-        <v>48.52199935913086</v>
+        <v>51.52999877929688</v>
       </c>
       <c r="C29" t="n">
-        <v>0.1904037147760391</v>
+        <v>0.1805908381938934</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1982</v>
+        <v>1983</v>
       </c>
       <c r="B30" t="n">
-        <v>51.52999877929688</v>
+        <v>53.55400085449219</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1805908381938934</v>
+        <v>0.1715885400772095</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1983</v>
+        <v>1984</v>
       </c>
       <c r="B31" t="n">
-        <v>53.55400085449219</v>
+        <v>55.45899963378906</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1715885400772095</v>
+        <v>0.1866784542798996</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1984</v>
+        <v>1985</v>
       </c>
       <c r="B32" t="n">
-        <v>55.45899963378906</v>
+        <v>57.23600006103516</v>
       </c>
       <c r="C32" t="n">
-        <v>0.1866784542798996</v>
+        <v>0.1689666360616684</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1985</v>
+        <v>1986</v>
       </c>
       <c r="B33" t="n">
-        <v>57.23600006103516</v>
+        <v>58.39300155639648</v>
       </c>
       <c r="C33" t="n">
-        <v>0.1689666360616684</v>
+        <v>0.1678354144096375</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1986</v>
+        <v>1987</v>
       </c>
       <c r="B34" t="n">
-        <v>58.39300155639648</v>
+        <v>59.87900161743164</v>
       </c>
       <c r="C34" t="n">
-        <v>0.1678354144096375</v>
+        <v>0.1611267477273941</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1987</v>
+        <v>1988</v>
       </c>
       <c r="B35" t="n">
-        <v>59.87900161743164</v>
+        <v>61.9739990234375</v>
       </c>
       <c r="C35" t="n">
-        <v>0.1611267477273941</v>
+        <v>0.1606961488723755</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1988</v>
+        <v>1989</v>
       </c>
       <c r="B36" t="n">
-        <v>61.9739990234375</v>
+        <v>64.38800048828125</v>
       </c>
       <c r="C36" t="n">
-        <v>0.1606961488723755</v>
+        <v>0.1732148230075836</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1989</v>
+        <v>1990</v>
       </c>
       <c r="B37" t="n">
-        <v>64.38800048828125</v>
+        <v>66.77400207519531</v>
       </c>
       <c r="C37" t="n">
-        <v>0.1732148230075836</v>
+        <v>0.163935050368309</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1990</v>
+        <v>1991</v>
       </c>
       <c r="B38" t="n">
-        <v>66.77400207519531</v>
+        <v>68.99299621582031</v>
       </c>
       <c r="C38" t="n">
-        <v>0.163935050368309</v>
+        <v>0.1436435878276825</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="B39" t="n">
-        <v>68.99299621582031</v>
+        <v>70.56400299072266</v>
       </c>
       <c r="C39" t="n">
-        <v>0.1436435878276825</v>
+        <v>0.1324461400508881</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="B40" t="n">
-        <v>70.56400299072266</v>
+        <v>72.24400329589844</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1324461400508881</v>
+        <v>0.1264168173074722</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="B41" t="n">
-        <v>72.24400329589844</v>
+        <v>73.78099822998047</v>
       </c>
       <c r="C41" t="n">
-        <v>0.1264168173074722</v>
+        <v>0.1407416164875031</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="B42" t="n">
-        <v>73.78099822998047</v>
+        <v>75.32099914550781</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1407416164875031</v>
+        <v>0.157494068145752</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="B43" t="n">
-        <v>75.32099914550781</v>
+        <v>76.69499969482422</v>
       </c>
       <c r="C43" t="n">
-        <v>0.157494068145752</v>
+        <v>0.1547413915395737</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="B44" t="n">
-        <v>76.69499969482422</v>
+        <v>78.00900268554688</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1547413915395737</v>
+        <v>0.1574671566486359</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="B45" t="n">
-        <v>78.00900268554688</v>
+        <v>78.85500335693359</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1574671566486359</v>
+        <v>0.1626884192228317</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="B46" t="n">
-        <v>78.85500335693359</v>
+        <v>80.06099700927734</v>
       </c>
       <c r="C46" t="n">
-        <v>0.1626884192228317</v>
+        <v>0.1544061899185181</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="B47" t="n">
-        <v>80.06099700927734</v>
+        <v>81.88300323486328</v>
       </c>
       <c r="C47" t="n">
-        <v>0.1544061899185181</v>
+        <v>0.1596006006002426</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="B48" t="n">
-        <v>81.88300323486328</v>
+        <v>83.75299835205078</v>
       </c>
       <c r="C48" t="n">
-        <v>0.1596006006002426</v>
+        <v>0.136037603020668</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B49" t="n">
-        <v>83.75299835205078</v>
+        <v>85.03800201416016</v>
       </c>
       <c r="C49" t="n">
-        <v>0.136037603020668</v>
+        <v>0.1213238909840584</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="B50" t="n">
-        <v>85.03800201416016</v>
+        <v>86.72899627685547</v>
       </c>
       <c r="C50" t="n">
-        <v>0.1213238909840584</v>
+        <v>0.1113898381590843</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="B51" t="n">
-        <v>86.72899627685547</v>
+        <v>89.11399841308594</v>
       </c>
       <c r="C51" t="n">
-        <v>0.1113898381590843</v>
+        <v>0.1059921905398369</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="B52" t="n">
-        <v>89.11399841308594</v>
+        <v>91.98100280761719</v>
       </c>
       <c r="C52" t="n">
-        <v>0.1059921905398369</v>
+        <v>0.1199610084295273</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="B53" t="n">
-        <v>91.98100280761719</v>
+        <v>94.81199645996094</v>
       </c>
       <c r="C53" t="n">
-        <v>0.1199610084295273</v>
+        <v>0.1388636380434036</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="B54" t="n">
-        <v>94.81199645996094</v>
+        <v>97.33399963378906</v>
       </c>
       <c r="C54" t="n">
-        <v>0.1388636380434036</v>
+        <v>0.1435916274785995</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B55" t="n">
-        <v>97.33399963378906</v>
+        <v>99.25</v>
       </c>
       <c r="C55" t="n">
-        <v>0.1435916274785995</v>
+        <v>0.119590200483799</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B56" t="n">
-        <v>99.25</v>
+        <v>100</v>
       </c>
       <c r="C56" t="n">
-        <v>0.119590200483799</v>
+        <v>0.1140433251857758</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B57" t="n">
-        <v>100</v>
+        <v>101.2170028686523</v>
       </c>
       <c r="C57" t="n">
-        <v>0.1140433251857758</v>
+        <v>0.109579972922802</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="B58" t="n">
-        <v>101.2170028686523</v>
+        <v>103.306999206543</v>
       </c>
       <c r="C58" t="n">
-        <v>0.109579972922802</v>
+        <v>0.1003680005669594</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B59" t="n">
-        <v>103.306999206543</v>
+        <v>105.2129974365234</v>
       </c>
       <c r="C59" t="n">
-        <v>0.1003680005669594</v>
+        <v>0.1029501557350159</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B60" t="n">
-        <v>105.2129974365234</v>
+        <v>106.9100036621094</v>
       </c>
       <c r="C60" t="n">
-        <v>0.1029501557350159</v>
+        <v>0.1049457564949989</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="B61" t="n">
-        <v>106.9100036621094</v>
+        <v>108.822998046875</v>
       </c>
       <c r="C61" t="n">
-        <v>0.1049457564949989</v>
+        <v>0.1029981672763824</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B62" t="n">
-        <v>108.822998046875</v>
+        <v>110.0100021362305</v>
       </c>
       <c r="C62" t="n">
-        <v>0.1029981672763824</v>
+        <v>0.1029981970787048</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B63" t="n">
-        <v>110.0100021362305</v>
+        <v>111.4120025634766</v>
       </c>
       <c r="C63" t="n">
         <v>0.1029981970787048</v>
@@ -1127,65 +1129,65 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B64" t="n">
-        <v>111.4120025634766</v>
+        <v>113.38653</v>
       </c>
       <c r="C64" t="n">
-        <v>0.1029981970787048</v>
+        <v>0.1110426258225217</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B65" t="n">
-        <v>113.38653</v>
+        <v>116.11404</v>
       </c>
       <c r="C65" t="n">
-        <v>0.1110426258225217</v>
+        <v>0.1142616929409515</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B66" t="n">
-        <v>116.11404</v>
+        <v>118.19775</v>
       </c>
       <c r="C66" t="n">
-        <v>0.1142616929409515</v>
+        <v>0.123637958252077</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B67" t="n">
-        <v>118.19775</v>
+        <v>119.72764</v>
       </c>
       <c r="C67" t="n">
-        <v>0.123637958252077</v>
+        <v>0.1108148551368363</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B68" t="n">
-        <v>119.72764</v>
+        <v>125.09162</v>
       </c>
       <c r="C68" t="n">
-        <v>0.1108148551368363</v>
+        <v>0.0759984821549977</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B69" t="n">
-        <v>125.09162</v>
+        <v>134.61324</v>
       </c>
       <c r="C69" t="n">
         <v>0.0759984821549977</v>
@@ -1193,43 +1195,36 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B70" t="n">
-        <v>134.61324</v>
+        <v>138.1988594658687</v>
       </c>
       <c r="C70" t="n">
-        <v>0.0759984821549977</v>
+        <v>0.1125698674711047</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B71" t="n">
-        <v>138.1988594658687</v>
+        <v>141.631754277003</v>
       </c>
       <c r="C71" t="n">
-        <v>0.1125698674711047</v>
+        <v>0.1272597457142391</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B72" t="n">
-        <v>141.631754277003</v>
+        <v>147.1305797411608</v>
       </c>
       <c r="C72" t="n">
-        <v>0.1272597457142391</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
+        <v>0.1183909054962436</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>